<commit_message>
fix(F-NAR-008): leçon implicite (square, goût, tour de parole)
Plus de « il faut demander » / « il faut attendre » / « même leçon ».
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-01.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-01.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le nez rose d'Amir</t>
+          <t>Le petit pain d'Amir</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, classe, puis maison</t>
+          <t>boulangerie du village, vitrine farinée, batteur</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, papa, maman, maîtresse</t>
+          <t>Amir, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Une carotte sent encore la terre. Amir veut dire que le lapin a un nez rose. Il lève la main, il attend, puis il le dit et le dessine.</t>
+          <t>Amir veut le petit pain rond au grain de sucre. Il parle trop tôt. Le batteur couvre sa voix. Il lève la main, il attend, puis maman l'entend.</t>
         </is>
       </c>
     </row>
@@ -1189,12 +1189,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un sac en papier craque sur la table. Dedans, une carotte sent encore la terre. Un peu de terre est sur le carreau. Une chaussette blanche a une oreille de lapin. Le jardin, derrière la porte, sent l'herbe mouillée. La carotte est pour plus tard, Amir. Le lapin du livre a un nez rose. Tout petit. Tu pourras le dire à l'école. Tu attends ton tour, d'accord ? D'accord, papa. Le cartable est un peu lourd. Tu vas bien t'asseoir ? Oui, maman. En ce moment, Amir arrive en classe. Le tapis est gris, un peu rêche. Au revoir, Amir. Bonne journée. Au revoir, maman. Amir s'assoit sur le tapis. Ses pieds restent bien posés. Une feuille jaune est collée sous une chaussure. Le vent pousse encore les arbres du jardin. La maîtresse montre une image. C'est un lapin blanc. Les oreilles sont trop longues. Le nez est rose, tout petit. On écoute d'abord l'image. Qui veut parler du lapin ? Amir a une idée. Le nez est rose, comme une gomme. Les mots lui chatouillent la bouche. Je veux parler du nez.</t>
+          <t>La farine poudre le rebord de la vitrine. Ça sent le beurre chaud, très fort. Un batteur tourne derrière le bois. Il fait un gros rrrr, tout grave. Des grains de sucre brillent sur un plateau. Tu as vu les petits ronds, Amir ? Oui. Celui-là a un grain de sucre. Je le veux. On va le dire, alors. En ce moment, maman parle vers le bois. Sa voix se mêle au batteur. Amir a les mots tout prêts. Le petit rond ! Avec le sucre ! Les mots tombent dans le rrrr. Personne ne se tourne. Le plateau reste loin, derrière la vitre. Maman. Maman parle encore, un peu plus fort. Amir ferme la bouche. Il lève la main, tout droit. Sa main reste en l'air, près du bois. Le batteur tourne, tourne. Puis il s'arrête. Le silence est tout chaud, tout soudain. Maman se tourne. Tu voulais dire quelque chose ? Le petit rond. Avec le grain de sucre. Je t'entends, maintenant. Une pince prend le pain doré. Le sachet craque, un peu gras. C'est lui. Merci, Amir. Tu as attendu, et je t'ai entendu. Le grain de sucre brille encore. Amir le garde du doigt, à travers le papier. On le mange sur le pas de la porte ? Oui.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sami arrive en classe avec maman. Maman dit au revoir. Sami s'assoit sur le tapis. La maîtresse pose une question. Sami a une idée. Il lève la main. Il faut &lt;emphasis level="moderate"&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Sami attend encore. Puis la maîtresse dit : Sami, c'est ton tour. Sami parle. Il dit : le lapin est blanc. La maîtresse sourit. Le soir, maman demande. Sami dit : j'ai levé la main. J'ai su attendre. Puis j'ai parlé.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>La farine poudre le rebord de la vitrine. Ça sent le beurre chaud, très fort. Un batteur tourne derrière le bois. Il fait un gros rrrr, tout grave. Des grains de sucre brillent sur un plateau. Tu as vu les petits ronds, Amir ? Oui. Celui-là a un grain de sucre. Je le veux. On va le dire, alors. En ce moment, maman parle vers le bois. Sa voix se mêle au batteur. Amir a les mots tout prêts. Le petit rond ! Avec le sucre ! Les mots tombent dans le rrrr. Personne ne se tourne. Le plateau reste loin, derrière la vitre. Maman. Maman parle encore, un peu plus fort. Amir ferme la bouche. Il lève la main, tout droit. Sa main reste en l'air, près du bois. Le batteur tourne, tourne. Puis il s'arrête. Le silence est tout chaud, tout soudain. Maman se tourne. Tu voulais dire quelque chose ? Le petit rond. Avec le grain de sucre. Je t'entends, maintenant. Une pince prend le pain doré. Le sachet craque, un peu gras. C'est lui. Merci, Amir. Tu as attendu, et je t'ai entendu. Le grain de sucre brille encore. Amir le garde du doigt, à travers le papier. On le mange sur le pas de la porte ? Oui.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1329,39 +1329,46 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un sac en papier craque sur la table.
-narrateur|Dedans, une carotte sent encore la terre.
-narrateur|Un peu de terre est sur le carreau.
-narrateur|Une chaussette blanche a une oreille de lapin.
-narrateur|Le jardin, derrière la porte, sent l'herbe mouillée.
-maman|La carotte est pour plus tard, Amir.
-enfant-m|Le lapin du livre a un nez rose.
-enfant-m|Tout petit.
-papa|Tu pourras le dire à l'école.
-papa|Tu attends ton tour, d'accord ?
-enfant-m|D'accord, papa.
-maman|Le cartable est un peu lourd.
-maman|Tu vas bien t'asseoir ?
-enfant-m|Oui, maman.
-narrateur|En ce moment, Amir arrive en classe.
-narrateur|Le tapis est gris, un peu rêche.
-maman|Au revoir, Amir.
-maman|Bonne journée.
-enfant-m|Au revoir, maman.
-narrateur|Amir s'assoit sur le tapis.
-narrateur|Ses pieds restent bien posés.
-narrateur|Une feuille jaune est collée sous une chaussure.
-narrateur|Le vent pousse encore les arbres du jardin.
-narrateur|La maîtresse montre une image.
-narrateur|C'est un lapin blanc.
-narrateur|Les oreilles sont trop longues.
-narrateur|Le nez est rose, tout petit.
-maitresse|On écoute d'abord l'image.
-maitresse|Qui veut parler du lapin ?
-narrateur|Amir a une idée.
-narrateur|Le nez est rose, comme une gomme.
-narrateur|Les mots lui chatouillent la bouche.
-enfant-m|Je veux parler du nez.</t>
+          <t>narrateur|La farine poudre le rebord de la vitrine.
+narrateur|Ça sent le beurre chaud, très fort.
+narrateur|Un batteur tourne derrière le bois.
+narrateur|Il fait un gros rrrr, tout grave.
+narrateur|Des grains de sucre brillent sur un plateau.
+maman|Tu as vu les petits ronds, Amir ?
+enfant-m|Oui.
+enfant-m|Celui-là a un grain de sucre.
+enfant-m|Je le veux.
+maman|On va le dire, alors.
+narrateur|En ce moment, maman parle vers le bois.
+narrateur|Sa voix se mêle au batteur.
+narrateur|Amir a les mots tout prêts.
+enfant-m|Le petit rond !
+enfant-m|Avec le sucre !
+narrateur|Les mots tombent dans le rrrr.
+narrateur|Personne ne se tourne.
+narrateur|Le plateau reste loin, derrière la vitre.
+enfant-m|Maman.
+narrateur|Maman parle encore, un peu plus fort.
+narrateur|Amir ferme la bouche.
+narrateur|Il lève la main, tout droit.
+narrateur|Sa main reste en l'air, près du bois.
+narrateur|Le batteur tourne, tourne.
+narrateur|Puis il s'arrête.
+narrateur|Le silence est tout chaud, tout soudain.
+narrateur|Maman se tourne.
+maman|Tu voulais dire quelque chose ?
+enfant-m|Le petit rond.
+enfant-m|Avec le grain de sucre.
+maman|Je t'entends, maintenant.
+narrateur|Une pince prend le pain doré.
+narrateur|Le sachet craque, un peu gras.
+enfant-m|C'est lui.
+maman|Merci, Amir.
+maman|Tu as attendu, et je t'ai entendu.
+narrateur|Le grain de sucre brille encore.
+narrateur|Amir le garde du doigt, à travers le papier.
+maman|On le mange sur le pas de la porte ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1398,7 +1405,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sami veut parler. Que fait-il d'abord ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>Amir veut parler. Que fait-il d'abord ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1428,7 +1435,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il lève la main et il attend. Que fait Amir ?</t>
+          <t>Personne ne l'entend. Que fait Amir d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1477,7 +1484,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.28</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1577,12 +1584,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir lève la main. Sa main reste en l'air. Il faut attendre. Il attend. Quelqu'un parle d'abord. On entend parler des oreilles. Amir attend encore. Il regarde le petit nez rose. Amir, c'est ton tour. Amir parle, tout doucement. Le lapin a un nez rose. Tout petit. Merci, Amir. Tu as attendu. Puis tu as parlé. Tu veux dessiner le nez ? Oui. Amir prend un crayon rose. Le crayon sent un peu le bois. Il fait un point, tout rond. Le point est trop gros, d'abord. Il le frotte un peu, tout doux. Le lapin a son nez, sur le papier. Le nez est bien là.</t>
+          <t>Le pas de la porte est tiède. Amir ouvre le sachet. Le pain est encore chaud dans la paume. Le grain de sucre est là. Tu le croques ? Oui. Le sucre casse, tout fin. La mie est blanche, un peu filante. Tu m'as entendu. Oui. Quand le batteur s'est tu. Quand ta main était là. Une miette tombe sur la farine du rebord. Amir la pousse du doigt, tout doux. Il est bon ? Il est chaud. Le village sent le pain, tout entier. Le sachet vide reste un peu gras.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sami a levé la main. Il a attendu. &lt;emphasis level="moderate"&gt;puis&lt;/emphasis&gt; il a parlé. C'était son tour.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le pas de la porte est tiède. Amir ouvre le sachet. Le pain est encore chaud dans la paume. Le grain de sucre est là. Tu le croques ? Oui. Le sucre casse, tout fin. La mie est blanche, un peu filante. Tu m'as entendu. Oui. Quand le batteur s'est tu. Quand ta main était là. Une miette tombe sur la farine du rebord. Amir la pousse du doigt, tout doux. Il est bon ? Il est chaud. Le village sent le pain, tout entier. Le sachet vide reste un peu gras.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1721,30 +1728,24 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir lève la main.
-narrateur|Sa main reste en l'air.
-narrateur|Il faut attendre.
-narrateur|Il attend.
-narrateur|Quelqu'un parle d'abord.
-narrateur|On entend parler des oreilles.
-narrateur|Amir attend encore.
-narrateur|Il regarde le petit nez rose.
-maitresse|Amir, c'est ton tour.
-narrateur|Amir parle, tout doucement.
-enfant-m|Le lapin a un nez rose.
-enfant-m|Tout petit.
-maitresse|Merci, Amir.
-maitresse|Tu as attendu.
-maitresse|Puis tu as parlé.
-maitresse|Tu veux dessiner le nez ?
+          <t>narrateur|Le pas de la porte est tiède.
+narrateur|Amir ouvre le sachet.
+narrateur|Le pain est encore chaud dans la paume.
+enfant-m|Le grain de sucre est là.
+maman|Tu le croques ?
 enfant-m|Oui.
-narrateur|Amir prend un crayon rose.
-narrateur|Le crayon sent un peu le bois.
-narrateur|Il fait un point, tout rond.
-narrateur|Le point est trop gros, d'abord.
-narrateur|Il le frotte un peu, tout doux.
-narrateur|Le lapin a son nez, sur le papier.
-maitresse|Le nez est bien là.</t>
+narrateur|Le sucre casse, tout fin.
+narrateur|La mie est blanche, un peu filante.
+enfant-m|Tu m'as entendu.
+maman|Oui.
+maman|Quand le batteur s'est tu.
+maman|Quand ta main était là.
+narrateur|Une miette tombe sur la farine du rebord.
+narrateur|Amir la pousse du doigt, tout doux.
+maman|Il est bon ?
+enfant-m|Il est chaud.
+narrateur|Le village sent le pain, tout entier.
+narrateur|Le sachet vide reste un peu gras.</t>
         </is>
       </c>
     </row>
@@ -1771,12 +1772,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le soir, maman ouvre la porte. La fermeture du cartable fait un petit zzz. Alors, Amir ? J'ai dit le nez rose. Il est sur le papier. Tu montres ? Oui, papa. Le point rose est un peu fort. Il est bien là. La carotte est encore dans le sac. Tu la croques en chemin ? Oui. Tu mets ton manteau ? Oui, maman. Le manteau sent le jardin.</t>
+          <t>Maman essuie un grain de farine. Il était sur la joue d'Amir. On rentre ? Oui. J'ai eu le petit rond. Oui. Je t'ai entendu. Le batteur reprend, plus loin, plus bas. Amir lèche un peu de sucre au pouce. Il en reste ? Un tout petit peu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sami range son cartable. Maman l'attend à la porte.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Maman essuie un grain de farine. Il était sur la joue d'Amir. On rentre ? Oui. J'ai eu le petit rond. Oui. Je t'ai entendu. Le batteur reprend, plus loin, plus bas. Amir lèche un peu de sucre au pouce. Il en reste ? Un tout petit peu.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1907,21 +1908,17 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Le soir, maman ouvre la porte.
-narrateur|La fermeture du cartable fait un petit zzz.
-maman|Alors, Amir ?
-enfant-m|J'ai dit le nez rose.
-enfant-m|Il est sur le papier.
-papa|Tu montres ?
-enfant-m|Oui, papa.
-narrateur|Le point rose est un peu fort.
-maman|Il est bien là.
-papa|La carotte est encore dans le sac.
-papa|Tu la croques en chemin ?
+          <t>narrateur|Maman essuie un grain de farine.
+narrateur|Il était sur la joue d'Amir.
+maman|On rentre ?
 enfant-m|Oui.
-maman|Tu mets ton manteau ?
-enfant-m|Oui, maman.
-narrateur|Le manteau sent le jardin.</t>
+enfant-m|J'ai eu le petit rond.
+maman|Oui.
+maman|Je t'ai entendu.
+narrateur|Le batteur reprend, plus loin, plus bas.
+narrateur|Amir lèche un peu de sucre au pouce.
+maman|Il en reste ?
+enfant-m|Un tout petit peu.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1953,12 +1950,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le nez rose est sur le papier. J'ai levé la main. J'ai attendu. Puis j'ai parlé. Bravo, Amir.</t>
+          <t>Le sachet craque encore dans la poche. Tu m'as entendu. Oui. Un grain de sucre brille sur le pouce. La vitrine reste poudreuse, calme.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le nez rose est sur le papier. J'ai levé la main. J'ai attendu. Puis j'ai parlé. Bravo, Amir.</t>
+          <t>Le sachet craque encore dans la poche. Tu m'as entendu. Oui. Un grain de sucre brille sur le pouce. La vitrine reste poudreuse, calme.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2014,14 +2011,14 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
         <v>0.88</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.22</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2093,11 +2090,11 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le nez rose est sur le papier.
-enfant-m|J'ai levé la main.
-enfant-m|J'ai attendu.
-enfant-m|Puis j'ai parlé.
-maman|Bravo, Amir.</t>
+          <t>narrateur|Le sachet craque encore dans la poche.
+enfant-m|Tu m'as entendu.
+maman|Oui.
+narrateur|Un grain de sucre brille sur le pouce.
+narrateur|La vitrine reste poudreuse, calme.</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2203,6 +2200,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-01 Le nez rose d'Amir
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-01.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-01.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le petit pain d'Amir</t>
+          <t>Le nez rose d'Amir</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>boulangerie du village, vitrine farinée, batteur</t>
+          <t>cuisine, classe, puis maison</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, maman</t>
+          <t>Amir, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut le petit pain rond au grain de sucre. Il parle trop tôt. Le batteur couvre sa voix. Il lève la main, il attend, puis maman l'entend.</t>
+          <t>Un sac en papier craque. Une carotte sent la terre. Sur la carotte, un éclat de carotte brille. Amir veut montrer le nez rose, maintenant. Il parle trop vite : les mots se perdent. Il lève le sac : personne ne regarde. Il refuse de foncer, lève la main, attend, puis dit. Merci vécu. Sur la table, l'éclat de carotte tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La farine poudre le rebord de la vitrine. Ça sent le beurre chaud, très fort. Un batteur tourne derrière le bois. Il fait un gros rrrr, tout grave. Des grains de sucre brillent sur un plateau. Tu as vu les petits ronds, Amir ? Oui. Celui-là a un grain de sucre. Je le veux. On va le dire, alors. En ce moment, maman parle vers le bois. Sa voix se mêle au batteur. Amir a les mots tout prêts. Le petit rond ! Avec le sucre ! Les mots tombent dans le rrrr. Personne ne se tourne. Le plateau reste loin, derrière la vitre. Maman. Maman parle encore, un peu plus fort. Amir ferme la bouche. Il lève la main, tout droit. Sa main reste en l'air, près du bois. Le batteur tourne, tourne. Puis il s'arrête. Le silence est tout chaud, tout soudain. Maman se tourne. Tu voulais dire quelque chose ? Le petit rond. Avec le grain de sucre. Je t'entends, maintenant. Une pince prend le pain doré. Le sachet craque, un peu gras. C'est lui. Merci, Amir. Tu as attendu, et je t'ai entendu. Le grain de sucre brille encore. Amir le garde du doigt, à travers le papier. On le mange sur le pas de la porte ? Oui.</t>
+          <t>La cuisine sent la terre, un peu. Un sac en papier craque sur la table. Dedans, une carotte sent la terre. Un peu de terre est sur le carreau. Une chaussette blanche a une oreille de lapin. Le jardin, derrière la porte, sent l'herbe mouillée. La carotte est pour plus tard, Amir. Le lapin du livre a un nez rose. Tout petit. Tu le montres à l'école ? Oui, papa. Sur la carotte, un éclat de carotte brille. Je le mets sur mon nez, maintenant ! En ce moment, Amir saisit la carotte. L'éclat de carotte saute près du sac. Le nez est rose, papa ! Papa n'a pas fini sa phrase. Les deux voix se mélangent. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas ! Ta main est trop vite ? Papa s'accroupit à la même hauteur. Amir parle trop fort, trop vite. Les mots se perdent près du sac. Oh. Ses épaules tombent un peu. Tes pieds sont sur le carreau ? Oui, papa. Ta chaussette blanche est à l'endroit ? Oui, maman. Tu vois l'oreille de lapin ? Oui. Elle est blanche. On la laisse sur la table ? Oui, elle est jolie. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le jardin sent l'herbe mouillée. Le sac en papier tape la hanche. La classe sent le papier et la pomme. La maîtresse parle près des chaises. Bonjour. Bonjour, maîtresse. Amir pose le sac près de sa chaise. Une image montre un lapin blanc. Les oreilles sont trop longues. Le nez est rose, tout petit. Les mots lui chatouillent la bouche. Je veux parler du nez. Plus tard, une voix s'approche. Elle parle des oreilles du lapin. Le nez est rose, maintenant ! Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Amir referme la bouche. Il repose les mains sur ses genoux. Le sac reste près de la chaise.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La farine poudre le rebord de la vitrine. Ça sent le beurre chaud, très fort. Un batteur tourne derrière le bois. Il fait un gros rrrr, tout grave. Des grains de sucre brillent sur un plateau. Tu as vu les petits ronds, Amir ? Oui. Celui-là a un grain de sucre. Je le veux. On va le dire, alors. En ce moment, maman parle vers le bois. Sa voix se mêle au batteur. Amir a les mots tout prêts. Le petit rond ! Avec le sucre ! Les mots tombent dans le rrrr. Personne ne se tourne. Le plateau reste loin, derrière la vitre. Maman. Maman parle encore, un peu plus fort. Amir ferme la bouche. Il lève la main, tout droit. Sa main reste en l'air, près du bois. Le batteur tourne, tourne. Puis il s'arrête. Le silence est tout chaud, tout soudain. Maman se tourne. Tu voulais dire quelque chose ? Le petit rond. Avec le grain de sucre. Je t'entends, maintenant. Une pince prend le pain doré. Le sachet craque, un peu gras. C'est lui. Merci, Amir. Tu as attendu, et je t'ai entendu. Le grain de sucre brille encore. Amir le garde du doigt, à travers le papier. On le mange sur le pas de la porte ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La cuisine sent la terre, un peu. Un sac en papier craque sur la table. Dedans, une carotte sent la terre. Un peu de terre est sur le carreau. Une chaussette blanche a une oreille de lapin. Le jardin, derrière la porte, sent l'herbe mouillée. La carotte est pour plus tard, Amir. Le lapin du livre a un nez rose. Tout petit. Tu le montres à l'école ? Oui, papa. Sur la carotte, un &lt;emphasis level="moderate"&gt;éclat de carotte&lt;/emphasis&gt; brille. Je le mets sur mon nez, maintenant ! En ce moment, Amir saisit la carotte. L'éclat de carotte saute près du sac. Le nez est rose, papa ! Papa n'a pas fini sa phrase. Les deux voix se mélangent. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas ! Ta main est trop vite ? Papa s'accroupit à la même hauteur. Amir parle trop fort, trop vite. Les mots se perdent près du sac. Oh. Ses épaules tombent un peu. Tes pieds sont sur le carreau ? Oui, papa. Ta chaussette blanche est à l'endroit ? Oui, maman. Tu vois l'oreille de lapin ? Oui. Elle est blanche. On la laisse sur la table ? Oui, elle est jolie. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le jardin sent l'herbe mouillée. Le sac en papier tape la hanche. La classe sent le papier et la pomme. La maîtresse parle près des chaises. Bonjour. Bonjour, maîtresse. Amir pose le sac près de sa chaise. Une image montre un lapin blanc. Les oreilles sont trop longues. Le nez est rose, tout petit. Les mots lui chatouillent la bouche. Je veux parler du nez. Plus tard, une voix s'approche. Elle parle des oreilles du lapin. Le nez est rose, maintenant ! Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Amir referme la bouche. Il repose les mains sur ses genoux. Le sac reste près de la chaise.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sami arrive en classe avec maman. Maman dit au revoir. Sami s'assoit sur le tapis. La maîtresse pose une question. Sami a une idée. Il lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Sami attend encore. Puis la maîtresse dit : Sami, c'est ton tour. Sami parle. Il dit : le lapin est blanc. La maîtresse sourit. Le soir, maman demande. Sami dit : j'ai levé la main. J'ai su attendre. Puis j'ai parlé. [pause]</t>
+          <t>La cuisine sent la terre, un peu. Un sac en papier craque sur la table. Dedans, une carotte sent la terre. Un peu de terre est sur le carreau. Une chaussette blanche a une oreille de lapin. Le jardin, derrière la porte, sent l'herbe mouillée. La carotte est pour plus tard, Amir. Le lapin du livre a un nez rose. Tout petit. Tu le montres à l'école ? Oui, papa. Sur la carotte, un &lt;emphasis&gt;éclat de carotte&lt;/emphasis&gt; brille. Je le mets sur mon nez, maintenant ! En ce moment, Amir saisit la carotte. L'éclat de carotte saute près du sac. Le nez est rose, papa ! Papa n'a pas fini sa phrase. Les deux voix se mélangent. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas ! Ta main est trop vite ? Papa s'accroupit à la même hauteur. Amir parle trop fort, trop vite. Les mots se perdent près du sac. Oh. Ses épaules tombent un peu. Tes pieds sont sur le carreau ? Oui, papa. Ta chaussette blanche est à l'endroit ? Oui, maman. Tu vois l'oreille de lapin ? Oui. Elle est blanche. On la laisse sur la table ? Oui, elle est jolie. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le jardin sent l'herbe mouillée. Le sac en papier tape la hanche. La classe sent le papier et la pomme. La maîtresse parle près des chaises. Bonjour. Bonjour, maîtresse. Amir pose le sac près de sa chaise. Une image montre un lapin blanc. Les oreilles sont trop longues. Le nez est rose, tout petit. Les mots lui chatouillent la bouche. Je veux parler du nez. Plus tard, une voix s'approche. Elle parle des oreilles du lapin. Le nez est rose, maintenant ! Ses mots se cognent à ceux de la classe. Personne ne tourne la tête. Amir referme la bouche. Il repose les mains sur ses genoux. Le sac reste près de la chaise. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de carotte</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,49 +1326,74 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_montrer_le_nez_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La farine poudre le rebord de la vitrine.
-narrateur|Ça sent le beurre chaud, très fort.
-narrateur|Un batteur tourne derrière le bois.
-narrateur|Il fait un gros rrrr, tout grave.
-narrateur|Des grains de sucre brillent sur un plateau.
-maman|Tu as vu les petits ronds, Amir ?
+          <t>narrateur|La cuisine sent la terre, un peu.
+narrateur|Un sac en papier craque sur la table.
+narrateur|Dedans, une carotte sent la terre.
+narrateur|Un peu de terre est sur le carreau.
+narrateur|Une chaussette blanche a une oreille de lapin.
+narrateur|Le jardin, derrière la porte, sent l'herbe mouillée.
+maman|La carotte est pour plus tard, Amir.
+enfant-m|Le lapin du livre a un nez rose.
+enfant-m|Tout petit.
+papa|Tu le montres à l'école ?
+enfant-m|Oui, papa.
+narrateur|Sur la carotte, un éclat de carotte brille.
+enfant-m|Je le mets sur mon nez, maintenant !
+narrateur|En ce moment, Amir saisit la carotte.
+narrateur|L'éclat de carotte saute près du sac.
+enfant-m|Le nez est rose, papa !
+narrateur|Papa n'a pas fini sa phrase.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Ça ne veut pas !
+papa|Ta main est trop vite ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Amir parle trop fort, trop vite.
+narrateur|Les mots se perdent près du sac.
+enfant-m|Oh.
+narrateur|Ses épaules tombent un peu.
+papa|Tes pieds sont sur le carreau ?
+enfant-m|Oui, papa.
+maman|Ta chaussette blanche est à l'endroit ?
+enfant-m|Oui, maman.
+papa|Tu vois l'oreille de lapin ?
 enfant-m|Oui.
-enfant-m|Celui-là a un grain de sucre.
-enfant-m|Je le veux.
-maman|On va le dire, alors.
-narrateur|En ce moment, maman parle vers le bois.
-narrateur|Sa voix se mêle au batteur.
-narrateur|Amir a les mots tout prêts.
-enfant-m|Le petit rond !
-enfant-m|Avec le sucre !
-narrateur|Les mots tombent dans le rrrr.
-narrateur|Personne ne se tourne.
-narrateur|Le plateau reste loin, derrière la vitre.
-enfant-m|Maman.
-narrateur|Maman parle encore, un peu plus fort.
-narrateur|Amir ferme la bouche.
-narrateur|Il lève la main, tout droit.
-narrateur|Sa main reste en l'air, près du bois.
-narrateur|Le batteur tourne, tourne.
-narrateur|Puis il s'arrête.
-narrateur|Le silence est tout chaud, tout soudain.
-narrateur|Maman se tourne.
-maman|Tu voulais dire quelque chose ?
-enfant-m|Le petit rond.
-enfant-m|Avec le grain de sucre.
-maman|Je t'entends, maintenant.
-narrateur|Une pince prend le pain doré.
-narrateur|Le sachet craque, un peu gras.
-enfant-m|C'est lui.
-maman|Merci, Amir.
-maman|Tu as attendu, et je t'ai entendu.
-narrateur|Le grain de sucre brille encore.
-narrateur|Amir le garde du doigt, à travers le papier.
-maman|On le mange sur le pas de la porte ?
-enfant-m|Oui.</t>
+enfant-m|Elle est blanche.
+maman|On la laisse sur la table ?
+enfant-m|Oui, elle est jolie.
+papa|On y va ?
+enfant-m|On y va.
+enfant-m|Au revoir, maman.
+maman|Au revoir, Amir.
+narrateur|Dehors, le jardin sent l'herbe mouillée.
+narrateur|Le sac en papier tape la hanche.
+narrateur|La classe sent le papier et la pomme.
+narrateur|La maîtresse parle près des chaises.
+maitresse|Bonjour.
+enfant-m|Bonjour, maîtresse.
+narrateur|Amir pose le sac près de sa chaise.
+narrateur|Une image montre un lapin blanc.
+narrateur|Les oreilles sont trop longues.
+narrateur|Le nez est rose, tout petit.
+narrateur|Les mots lui chatouillent la bouche.
+enfant-m|Je veux parler du nez.
+narrateur|Plus tard, une voix s'approche.
+narrateur|Elle parle des oreilles du lapin.
+enfant-m|Le nez est rose, maintenant !
+narrateur|Ses mots se cognent à ceux de la classe.
+narrateur|Personne ne tourne la tête.
+narrateur|Amir referme la bouche.
+narrateur|Il repose les mains sur ses genoux.
+narrateur|Le sac reste près de la chaise.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1405,37 +1430,37 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>attendre</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>attendre | il attend | lever la main | la main</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Oui, c'est la bonne réponse.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Tu étais presque.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
           <t>Amir veut parler. Que fait-il d'abord ?</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>&lt;slow&gt;Sami veut parler. Que fait-il d'abord ?&lt;/slow&gt;</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>attendre</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>attendre | il attend | lever la main | la main</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Oui, c'est la bonne réponse.</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Tu étais presque.</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Personne ne l'entend. Que fait Amir d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1473,7 +1498,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1484,7 +1509,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1499,34 +1524,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1541,17 +1570,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_leve_la_main_avant_de_parler; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1584,17 +1613,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le pas de la porte est tiède. Amir ouvre le sachet. Le pain est encore chaud dans la paume. Le grain de sucre est là. Tu le croques ? Oui. Le sucre casse, tout fin. La mie est blanche, un peu filante. Tu m'as entendu. Oui. Quand le batteur s'est tu. Quand ta main était là. Une miette tombe sur la farine du rebord. Amir la pousse du doigt, tout doux. Il est bon ? Il est chaud. Le village sent le pain, tout entier. Le sachet vide reste un peu gras.</t>
+          <t>Amir veut montrer la carotte, tout de suite. Il lève le sac trop vite. La carotte penche, puis retombe. Oh. Personne ne regarde le sac. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il lève la main. Sa main reste en l'air. Une autre voix parle des oreilles. Amir reste près de sa chaise. Il regarde le petit nez rose. L'éclat de carotte brille dans le sac. Amir. Un silence arrive, tout petit. Le lapin a un nez rose. Tout petit. Comme la carotte. Une tête se tourne vers lui. Les oreilles écoutent jusqu'au bout. Le soir, la porte s'ouvre. Ça sent la terre et le papier. Te voilà, Amir. Le sac est rentré. La carotte attend sur la table. La chaussette blanche est là. Amir regarde papa. Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le pas de la porte est tiède. Amir ouvre le sachet. Le pain est encore chaud dans la paume. Le grain de sucre est là. Tu le croques ? Oui. Le sucre casse, tout fin. La mie est blanche, un peu filante. Tu m'as entendu. Oui. Quand le batteur s'est tu. Quand ta main était là. Une miette tombe sur la farine du rebord. Amir la pousse du doigt, tout doux. Il est bon ? Il est chaud. Le village sent le pain, tout entier. Le sachet vide reste un peu gras.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut montrer la carotte, tout de suite. Il lève le sac trop vite. La carotte penche, puis retombe. Oh. Personne ne regarde le sac. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il lève la &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt;. Sa main reste en l'air. Une autre voix parle des oreilles. Amir reste près de sa chaise. Il regarde le petit nez rose. L'éclat de carotte brille dans le sac. Amir. Un silence arrive, tout petit. Le lapin a un nez rose. Tout petit. Comme la carotte. Une tête se tourne vers lui. Les oreilles écoutent jusqu'au bout. Le soir, la porte s'ouvre. Ça sent la terre et le papier. Te voilà, Amir. Le sac est rentré. La carotte attend sur la table. La chaussette blanche est là. Amir regarde papa. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sami a levé la main. Il a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; il a parlé. C'était son tour. [pause]</t>
+          <t>Amir veut montrer la carotte, tout de suite. Il lève le sac trop vite. La carotte penche, puis retombe. Oh. Personne ne regarde le sac. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il lève la &lt;emphasis&gt;main&lt;/emphasis&gt;. Sa main reste en l'air. Une autre voix parle des oreilles. Amir reste près de sa chaise. Il regarde le petit nez rose. L'éclat de carotte brille dans le sac. Amir. Un silence arrive, tout petit. Le lapin a un nez rose. Tout petit. Comme la carotte. Une tête se tourne vers lui. Les oreilles écoutent jusqu'au bout. Le soir, la porte s'ouvre. Ça sent la terre et le papier. Te voilà, Amir. Le sac est rentré. La carotte attend sur la table. La chaussette blanche est là. Amir regarde papa. Il ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1641,7 +1670,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1649,10 +1678,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1675,30 +1704,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>main</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1707,10 +1736,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1723,29 +1752,45 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_attend_puis_dit_le_nez_rose; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le pas de la porte est tiède.
-narrateur|Amir ouvre le sachet.
-narrateur|Le pain est encore chaud dans la paume.
-enfant-m|Le grain de sucre est là.
-maman|Tu le croques ?
-enfant-m|Oui.
-narrateur|Le sucre casse, tout fin.
-narrateur|La mie est blanche, un peu filante.
-enfant-m|Tu m'as entendu.
-maman|Oui.
-maman|Quand le batteur s'est tu.
-maman|Quand ta main était là.
-narrateur|Une miette tombe sur la farine du rebord.
-narrateur|Amir la pousse du doigt, tout doux.
-maman|Il est bon ?
-enfant-m|Il est chaud.
-narrateur|Le village sent le pain, tout entier.
-narrateur|Le sachet vide reste un peu gras.</t>
+          <t>narrateur|Amir veut montrer la carotte, tout de suite.
+narrateur|Il lève le sac trop vite.
+narrateur|La carotte penche, puis retombe.
+enfant-m|Oh.
+narrateur|Personne ne regarde le sac.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Il lève la main.
+narrateur|Sa main reste en l'air.
+narrateur|Une autre voix parle des oreilles.
+narrateur|Amir reste près de sa chaise.
+narrateur|Il regarde le petit nez rose.
+narrateur|L'éclat de carotte brille dans le sac.
+maitresse|Amir.
+narrateur|Un silence arrive, tout petit.
+enfant-m|Le lapin a un nez rose.
+enfant-m|Tout petit.
+enfant-m|Comme la carotte.
+narrateur|Une tête se tourne vers lui.
+narrateur|Les oreilles écoutent jusqu'au bout.
+narrateur|Le soir, la porte s'ouvre.
+narrateur|Ça sent la terre et le papier.
+papa|Te voilà, Amir.
+maman|Le sac est rentré.
+narrateur|La carotte attend sur la table.
+narrateur|La chaussette blanche est là.
+narrateur|Amir regarde papa.
+narrateur|Il ouvre la bouche.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>chaise,voix</t>
         </is>
       </c>
     </row>
@@ -1772,17 +1817,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman essuie un grain de farine. Il était sur la joue d'Amir. On rentre ? Oui. J'ai eu le petit rond. Oui. Je t'ai entendu. Le batteur reprend, plus loin, plus bas. Amir lèche un peu de sucre au pouce. Il en reste ? Un tout petit peu.</t>
+          <t>Amir veut dire le nez, tout de suite. Papa, le nez rose. Papa n'a pas fini sa phrase. Le sac est sur la table, Amir. Les deux voix se mélangent. Oh. Amir refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes pieds sont près de la table ? Papa pose le sac contre le bois. La chaussette blanche est sous la chaise. Maman n'a pas fini non plus. Amir reste jusqu'au silence. Je peux te dire quelque chose ? Oui, nous t'écoutons. Le lapin a un nez rose. Tout petit, comme la carotte. Merci, Amir. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Amir veut poser l'éclat, tout de suite. Il le saisit trop vite. L'éclat glisse entre ses doigts. Oh. Amir s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose l'éclat plus lentement. Le nez d'Amir devient un peu rose. Il est rose, maman !</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman essuie un grain de farine. Il était sur la joue d'Amir. On rentre ? Oui. J'ai eu le petit rond. Oui. Je t'ai entendu. Le batteur reprend, plus loin, plus bas. Amir lèche un peu de sucre au pouce. Il en reste ? Un tout petit peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut dire le nez, tout de suite. Papa, le nez rose. Papa n'a pas fini sa phrase. Le sac est sur la table, Amir. Les deux voix se mélangent. Oh. Amir refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes pieds sont près de la table ? Papa pose le sac contre le bois. La chaussette blanche est sous la chaise. Maman n'a pas fini non plus. Amir reste jusqu'au silence. Je peux te dire quelque chose ? Oui, nous t'écoutons. Le lapin a un nez rose. Tout petit, comme la &lt;emphasis level="moderate"&gt;carotte&lt;/emphasis&gt;. Merci, Amir. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Amir veut poser l'éclat, tout de suite. Il le saisit trop vite. L'éclat glisse entre ses doigts. Oh. Amir s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose l'éclat plus lentement. Le nez d'Amir devient un peu rose. Il est rose, maman !&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sami range son cartable. Maman l'attend à la porte. [pause]</t>
+          <t>Amir veut dire le nez, tout de suite. Papa, le nez rose. Papa n'a pas fini sa phrase. Le sac est sur la table, Amir. Les deux voix se mélangent. Oh. Amir refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes pieds sont près de la table ? Papa pose le sac contre le bois. La chaussette blanche est sous la chaise. Maman n'a pas fini non plus. Amir reste jusqu'au silence. Je peux te dire quelque chose ? Oui, nous t'écoutons. Le lapin a un nez rose. Tout petit, comme la &lt;emphasis&gt;carotte&lt;/emphasis&gt;. Merci, Amir. Papa a entendu toute la phrase. Tu veux un peu d'eau ? Oui, maman. Amir veut poser l'éclat, tout de suite. Il le saisit trop vite. L'éclat glisse entre ses doigts. Oh. Amir s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose l'éclat plus lentement. Le nez d'Amir devient un peu rose. Il est rose, maman ! [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1829,7 +1874,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1837,10 +1882,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1861,28 +1906,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>carotte</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1891,10 +1940,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1905,25 +1954,50 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_couper_papa; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman essuie un grain de farine.
-narrateur|Il était sur la joue d'Amir.
-maman|On rentre ?
-enfant-m|Oui.
-enfant-m|J'ai eu le petit rond.
-maman|Oui.
-maman|Je t'ai entendu.
-narrateur|Le batteur reprend, plus loin, plus bas.
-narrateur|Amir lèche un peu de sucre au pouce.
-maman|Il en reste ?
-enfant-m|Un tout petit peu.</t>
+          <t>narrateur|Amir veut dire le nez, tout de suite.
+enfant-m|Papa, le nez rose.
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le sac est sur la table, Amir.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Il pose les mains à plat.
+papa|Tes pieds sont près de la table ?
+narrateur|Papa pose le sac contre le bois.
+maman|La chaussette blanche est sous la chaise.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Amir reste jusqu'au silence.
+enfant-m|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-m|Le lapin a un nez rose.
+enfant-m|Tout petit, comme la carotte.
+papa|Merci, Amir.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu veux un peu d'eau ?
+enfant-m|Oui, maman.
+narrateur|Amir veut poser l'éclat, tout de suite.
+narrateur|Il le saisit trop vite.
+narrateur|L'éclat glisse entre ses doigts.
+enfant-m|Oh.
+narrateur|Amir s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il refuse de foncer.
+narrateur|Il pose l'éclat plus lentement.
+narrateur|Le nez d'Amir devient un peu rose.
+enfant-m|Il est rose, maman !</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte,manteau</t>
+          <t>table,eau</t>
         </is>
       </c>
     </row>
@@ -1950,17 +2024,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le sachet craque encore dans la poche. Tu m'as entendu. Oui. Un grain de sucre brille sur le pouce. La vitrine reste poudreuse, calme.</t>
+          <t>Ils restent près de la table. La carotte repose dans le sac. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la carotte. On est bien, ici. Le sac sent la terre, un peu. Amir glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. La chaussette blanche repose contre le bois. Elle a une oreille de lapin. On la laisse ? Oui. L'éclat de carotte tient sur la table.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le sachet craque encore dans la poche. Tu m'as entendu. Oui. Un grain de sucre brille sur le pouce. La vitrine reste poudreuse, calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. La carotte repose dans le sac. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la carotte. On est bien, ici. Le sac sent la terre, un peu. Amir glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. La chaussette blanche repose contre le bois. Elle a une oreille de lapin. On la laisse ? Oui. L'&lt;emphasis level="moderate"&gt;éclat de carotte&lt;/emphasis&gt; tient sur la table.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. La carotte repose dans le sac. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la carotte. On est bien, ici. Le sac sent la terre, un peu. Amir glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est frais. La chaussette blanche repose contre le bois. Elle a une oreille de lapin. On la laisse ? Oui. L'&lt;emphasis&gt;éclat de carotte&lt;/emphasis&gt; tient sur la table.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,18 +2081,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2027,12 +2101,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2115,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de carotte</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2138,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,28 +2151,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_table; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le sachet craque encore dans la poche.
-enfant-m|Tu m'as entendu.
-maman|Oui.
-narrateur|Un grain de sucre brille sur le pouce.
-narrateur|La vitrine reste poudreuse, calme.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|La carotte repose dans le sac.
+enfant-m|Comme ce matin, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur la carotte.
+maman|On est bien, ici.
+narrateur|Le sac sent la terre, un peu.
+narrateur|Amir glisse le pied, sans se presser.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes joues ?
+enfant-m|Oui, il est frais.
+narrateur|La chaussette blanche repose contre le bois.
+enfant-m|Elle a une oreille de lapin.
+papa|On la laisse ?
+enfant-m|Oui.
+narrateur|L'éclat de carotte tient sur la table.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>sac,carotte</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2207,6 +2305,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>